<commit_message>
added logout, venue_admin app with accept and decline option
</commit_message>
<xml_diff>
--- a/user_info.xlsx
+++ b/user_info.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="41">
   <si>
     <t>name</t>
   </si>
@@ -73,7 +73,7 @@
     <t>None</t>
   </si>
   <si>
-    <t>faculty_advisor</t>
+    <t>Faculty</t>
   </si>
   <si>
     <t>mane</t>
@@ -93,6 +93,9 @@
     <t>SDS</t>
   </si>
   <si>
+    <t>faculty_advisor</t>
+  </si>
+  <si>
     <t>amit</t>
   </si>
   <si>
@@ -123,6 +126,71 @@
   <si>
     <t>Impressions</t>
   </si>
+  <si>
+    <t>AC</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u val="single"/>
+        <sz val="11"/>
+        <color indexed="11"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>ac.test@gmail.com</t>
+    </r>
+  </si>
+  <si>
+    <t>Venue_admin</t>
+  </si>
+  <si>
+    <t>Cognizant</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u val="single"/>
+        <sz val="11"/>
+        <color indexed="11"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>cognizant.test@gmail.com</t>
+    </r>
+  </si>
+  <si>
+    <t>Cognizant Lab</t>
+  </si>
+  <si>
+    <t>Foss</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u val="single"/>
+        <sz val="11"/>
+        <color indexed="11"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>foss.test@gmail.com</t>
+    </r>
+  </si>
+  <si>
+    <t>FOSS</t>
+  </si>
+  <si>
+    <t>Kiran</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u val="single"/>
+        <sz val="11"/>
+        <color indexed="11"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>impressions.fac.ad@gmail.com</t>
+    </r>
+  </si>
 </sst>
 </file>
 
@@ -131,7 +199,7 @@
   <numFmts count="1">
     <numFmt numFmtId="0" formatCode="General"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color indexed="8"/>
@@ -157,6 +225,11 @@
       <sz val="11"/>
       <color indexed="11"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="8"/>
+      <name val="Menlo Regular"/>
     </font>
   </fonts>
   <fills count="3">
@@ -218,8 +291,8 @@
     <xf numFmtId="49" fontId="0" fillId="2" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
+    <xf numFmtId="49" fontId="5" fillId="2" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment horizontal="left" vertical="bottom" readingOrder="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -393,7 +466,7 @@
           <a:effectLst>
             <a:outerShdw sx="100000" sy="100000" kx="0" ky="0" algn="b" rotWithShape="0" blurRad="38100" dist="23000" dir="5400000">
               <a:srgbClr val="000000">
-                <a:alpha val="38000"/>
+                <a:alpha val="35000"/>
               </a:srgbClr>
             </a:outerShdw>
           </a:effectLst>
@@ -473,7 +546,7 @@
         </a:effectLst>
         <a:sp3d/>
       </a:spPr>
-      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="45719" tIns="45719" rIns="45719" bIns="45719" numCol="1" spcCol="38100" rtlCol="0" anchor="ctr" upright="0">
+      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="45718" tIns="45718" rIns="45718" bIns="45718" numCol="1" spcCol="38100" rtlCol="0" anchor="ctr" upright="0">
         <a:spAutoFit/>
       </a:bodyPr>
       <a:lstStyle>
@@ -500,10 +573,10 @@
             </a:solidFill>
             <a:effectLst/>
             <a:uFillTx/>
-            <a:latin typeface="Calibri"/>
-            <a:ea typeface="Calibri"/>
-            <a:cs typeface="Calibri"/>
-            <a:sym typeface="Calibri"/>
+            <a:latin typeface="+mn-lt"/>
+            <a:ea typeface="+mn-ea"/>
+            <a:cs typeface="+mn-cs"/>
+            <a:sym typeface="Helvetica Neue"/>
           </a:defRPr>
         </a:defPPr>
         <a:lvl1pPr marL="0" marR="0" indent="0" algn="l" defTabSz="914400" rtl="0" fontAlgn="auto" latinLnBrk="1" hangingPunct="0">
@@ -752,7 +825,7 @@
         <a:effectLst>
           <a:outerShdw sx="100000" sy="100000" kx="0" ky="0" algn="b" rotWithShape="0" blurRad="38100" dist="23000" dir="5400000">
             <a:srgbClr val="000000">
-              <a:alpha val="38000"/>
+              <a:alpha val="35000"/>
             </a:srgbClr>
           </a:outerShdw>
         </a:effectLst>
@@ -1030,7 +1103,7 @@
         <a:effectLst/>
         <a:sp3d/>
       </a:spPr>
-      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="45719" tIns="45719" rIns="45719" bIns="45719" numCol="1" spcCol="38100" rtlCol="0" anchor="t" upright="0">
+      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="45718" tIns="45718" rIns="45718" bIns="45718" numCol="1" spcCol="38100" rtlCol="0" anchor="t" upright="0">
         <a:spAutoFit/>
       </a:bodyPr>
       <a:lstStyle>
@@ -1057,10 +1130,10 @@
             </a:solidFill>
             <a:effectLst/>
             <a:uFillTx/>
-            <a:latin typeface="Calibri"/>
-            <a:ea typeface="Calibri"/>
-            <a:cs typeface="Calibri"/>
-            <a:sym typeface="Calibri"/>
+            <a:latin typeface="+mn-lt"/>
+            <a:ea typeface="+mn-ea"/>
+            <a:cs typeface="+mn-cs"/>
+            <a:sym typeface="Helvetica Neue"/>
           </a:defRPr>
         </a:defPPr>
         <a:lvl1pPr marL="0" marR="0" indent="0" algn="l" defTabSz="914400" rtl="0" fontAlgn="auto" latinLnBrk="1" hangingPunct="0">
@@ -1302,11 +1375,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr defaultColWidth="8.83333" defaultRowHeight="15" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="12.5" style="1" customWidth="1"/>
-    <col min="2" max="2" width="19.6719" style="1" customWidth="1"/>
+    <col min="2" max="2" width="32.5234" style="1" customWidth="1"/>
     <col min="3" max="3" width="16.6719" style="1" customWidth="1"/>
     <col min="4" max="4" width="15.6719" style="1" customWidth="1"/>
     <col min="5" max="6" width="12.5" style="1" customWidth="1"/>
@@ -1407,7 +1480,7 @@
         <v>15</v>
       </c>
       <c r="E5" t="s" s="2">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="F5" t="s" s="3">
         <v>10</v>
@@ -1415,10 +1488,10 @@
     </row>
     <row r="6" ht="13.65" customHeight="1">
       <c r="A6" t="s" s="4">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B6" t="s" s="4">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C6" t="s" s="4">
         <v>13</v>
@@ -1427,7 +1500,7 @@
         <v>14</v>
       </c>
       <c r="E6" t="s" s="2">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="F6" t="s" s="3">
         <v>10</v>
@@ -1435,13 +1508,13 @@
     </row>
     <row r="7" ht="13.65" customHeight="1">
       <c r="A7" t="s" s="4">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B7" t="s" s="4">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C7" t="s" s="4">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D7" t="s" s="4">
         <v>9</v>
@@ -1454,34 +1527,94 @@
       </c>
     </row>
     <row r="8" ht="13.55" customHeight="1">
-      <c r="A8" s="5"/>
-      <c r="B8" s="5"/>
-      <c r="C8" s="5"/>
-      <c r="D8" s="5"/>
-      <c r="E8" s="5"/>
-      <c r="F8" s="5"/>
+      <c r="A8" t="s" s="4">
+        <v>30</v>
+      </c>
+      <c r="B8" t="s" s="4">
+        <v>31</v>
+      </c>
+      <c r="C8" t="s" s="4">
+        <v>30</v>
+      </c>
+      <c r="D8" t="s" s="4">
+        <v>19</v>
+      </c>
+      <c r="E8" t="s" s="4">
+        <v>32</v>
+      </c>
+      <c r="F8" t="s" s="3">
+        <v>10</v>
+      </c>
     </row>
     <row r="9" ht="13.55" customHeight="1">
-      <c r="A9" s="5"/>
-      <c r="B9" s="5"/>
-      <c r="C9" s="5"/>
-      <c r="D9" s="5"/>
-      <c r="E9" s="5"/>
-      <c r="F9" s="5"/>
+      <c r="A9" t="s" s="4">
+        <v>33</v>
+      </c>
+      <c r="B9" t="s" s="4">
+        <v>34</v>
+      </c>
+      <c r="C9" t="s" s="5">
+        <v>35</v>
+      </c>
+      <c r="D9" t="s" s="4">
+        <v>19</v>
+      </c>
+      <c r="E9" t="s" s="4">
+        <v>32</v>
+      </c>
+      <c r="F9" t="s" s="3">
+        <v>10</v>
+      </c>
     </row>
     <row r="10" ht="13.55" customHeight="1">
-      <c r="A10" s="5"/>
-      <c r="B10" s="5"/>
-      <c r="C10" s="5"/>
-      <c r="D10" s="5"/>
-      <c r="E10" s="5"/>
-      <c r="F10" s="5"/>
+      <c r="A10" t="s" s="4">
+        <v>36</v>
+      </c>
+      <c r="B10" t="s" s="4">
+        <v>37</v>
+      </c>
+      <c r="C10" t="s" s="5">
+        <v>38</v>
+      </c>
+      <c r="D10" t="s" s="4">
+        <v>19</v>
+      </c>
+      <c r="E10" t="s" s="4">
+        <v>32</v>
+      </c>
+      <c r="F10" t="s" s="3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="11" ht="13.55" customHeight="1">
+      <c r="A11" t="s" s="4">
+        <v>39</v>
+      </c>
+      <c r="B11" t="s" s="4">
+        <v>40</v>
+      </c>
+      <c r="C11" t="s" s="5">
+        <v>29</v>
+      </c>
+      <c r="D11" t="s" s="4">
+        <v>9</v>
+      </c>
+      <c r="E11" t="s" s="2">
+        <v>24</v>
+      </c>
+      <c r="F11" t="s" s="3">
+        <v>10</v>
+      </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="B5" r:id="rId1" location="" tooltip="" display="mane.test@gmail.com"/>
     <hyperlink ref="B6" r:id="rId2" location="" tooltip="" display="amit.test@gmail.com"/>
     <hyperlink ref="B7" r:id="rId3" location="" tooltip="" display="idris.test@gmail.com"/>
+    <hyperlink ref="B8" r:id="rId4" location="" tooltip="" display="ac.test@gmail.com"/>
+    <hyperlink ref="B9" r:id="rId5" location="" tooltip="" display="cognizant.test@gmail.com"/>
+    <hyperlink ref="B10" r:id="rId6" location="" tooltip="" display="foss.test@gmail.com"/>
+    <hyperlink ref="B11" r:id="rId7" location="" tooltip="" display="impressions.fac.ad@gmail.com"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup firstPageNumber="1" fitToHeight="1" fitToWidth="1" scale="100" useFirstPageNumber="0" orientation="portrait" pageOrder="downThenOver"/>

</xml_diff>

<commit_message>
asynchronous email sending with threading
</commit_message>
<xml_diff>
--- a/user_info.xlsx
+++ b/user_info.xlsx
@@ -1,20 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion rupBuild="9303" lowestEdited="5" lastEdited="5" appName="xl"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29530"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Aasthami\Documents\GitHub\VenueBookingSystem\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E042163-7AA1-4444-A0D0-1CF373FCDAEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="0"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet r:id="rId1" sheetId="1" name="Sheet1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr fullCalcOnLoad="1"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="63">
   <si>
     <t>name</t>
   </si>
@@ -37,13 +43,10 @@
     <t>arnav</t>
   </si>
   <si>
-    <r>
-      <t/>
-    </r>
     <r>
       <rPr>
         <sz val="10"/>
-        <color rgb="FFff0000"/>
+        <color rgb="FFFF0000"/>
         <rFont val="Arial"/>
         <family val="2"/>
       </rPr>
@@ -67,12 +70,9 @@
   </si>
   <si>
     <r>
-      <t/>
-    </r>
-    <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFff0000"/>
+        <color rgb="FFFF0000"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -90,9 +90,6 @@
     <t>Abhishek_admin</t>
   </si>
   <si>
-    <r>
-      <t/>
-    </r>
     <r>
       <rPr>
         <sz val="11"/>
@@ -109,9 +106,6 @@
   </si>
   <si>
     <r>
-      <t/>
-    </r>
-    <r>
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
@@ -245,13 +239,18 @@
   <si>
     <t xml:space="preserve">Mr. Hrishikesh Kishor Jadhav </t>
   </si>
+  <si>
+    <t>Aastha</t>
+  </si>
+  <si>
+    <t>aastha.anuj.jajoo@gmail.com</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
-  <numFmts count="0"/>
-  <fonts count="5" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -267,7 +266,7 @@
     </font>
     <font>
       <sz val="10"/>
-      <color rgb="FFff0000"/>
+      <color rgb="FFFF0000"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -279,9 +278,31 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FFff0000"/>
+      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="4">
@@ -293,12 +314,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFffffff"/>
+        <fgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF00ff00"/>
+        <fgColor rgb="FF00FF00"/>
       </patternFill>
     </fill>
   </fills>
@@ -336,37 +357,37 @@
         <color rgb="FF000000"/>
       </top>
       <bottom style="thin">
-        <color rgb="FFffffff"/>
+        <color rgb="FFFFFFFF"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
       <left style="thin">
-        <color rgb="FFffffff"/>
+        <color rgb="FFFFFFFF"/>
       </left>
       <right style="thin">
-        <color rgb="FFffffff"/>
+        <color rgb="FFFFFFFF"/>
       </right>
       <top style="thin">
-        <color rgb="FFffffff"/>
+        <color rgb="FFFFFFFF"/>
       </top>
       <bottom style="thin">
-        <color rgb="FF00ff00"/>
+        <color rgb="FF00FF00"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
       <left style="thin">
-        <color rgb="FFffffff"/>
+        <color rgb="FFFFFFFF"/>
       </left>
       <right style="thin">
         <color rgb="FF000000"/>
       </right>
       <top style="thin">
-        <color rgb="FFffffff"/>
+        <color rgb="FFFFFFFF"/>
       </top>
       <bottom style="thin">
-        <color rgb="FF00ff00"/>
+        <color rgb="FF00FF00"/>
       </bottom>
       <diagonal/>
     </border>
@@ -375,43 +396,43 @@
         <color rgb="FF000000"/>
       </left>
       <right style="thin">
-        <color rgb="FF0000ff"/>
+        <color rgb="FF0000FF"/>
       </right>
       <top style="thin">
         <color rgb="FF000000"/>
       </top>
       <bottom style="thin">
-        <color rgb="FFc6c6c6"/>
+        <color rgb="FFC6C6C6"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
       <left style="thin">
-        <color rgb="FF00ff00"/>
+        <color rgb="FF00FF00"/>
       </left>
       <right style="thin">
-        <color rgb="FF00ff00"/>
+        <color rgb="FF00FF00"/>
       </right>
       <top style="thin">
-        <color rgb="FF00ff00"/>
+        <color rgb="FF00FF00"/>
       </top>
       <bottom style="thin">
-        <color rgb="FFffffff"/>
+        <color rgb="FFFFFFFF"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
       <left style="thin">
-        <color rgb="FF00ff00"/>
+        <color rgb="FF00FF00"/>
       </left>
       <right style="thin">
         <color rgb="FF000000"/>
       </right>
       <top style="thin">
-        <color rgb="FF00ff00"/>
+        <color rgb="FF00FF00"/>
       </top>
       <bottom style="thin">
-        <color rgb="FFffffff"/>
+        <color rgb="FFFFFFFF"/>
       </bottom>
       <diagonal/>
     </border>
@@ -420,106 +441,111 @@
         <color rgb="FF000000"/>
       </left>
       <right style="thin">
-        <color rgb="FF0000ff"/>
+        <color rgb="FF0000FF"/>
       </right>
       <top style="thin">
-        <color rgb="FFc6c6c6"/>
+        <color rgb="FFC6C6C6"/>
       </top>
       <bottom style="thin">
-        <color rgb="FFc6c6c6"/>
+        <color rgb="FFC6C6C6"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
       <left style="thin">
-        <color rgb="FFffffff"/>
+        <color rgb="FFFFFFFF"/>
       </left>
       <right style="thin">
-        <color rgb="FFffffff"/>
+        <color rgb="FFFFFFFF"/>
       </right>
       <top style="thin">
-        <color rgb="FFffffff"/>
+        <color rgb="FFFFFFFF"/>
       </top>
       <bottom style="thin">
-        <color rgb="FFffff00"/>
+        <color rgb="FFFFFF00"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
       <left style="thin">
-        <color rgb="FFffffff"/>
+        <color rgb="FFFFFFFF"/>
       </left>
       <right style="thin">
         <color rgb="FF000000"/>
       </right>
       <top style="thin">
-        <color rgb="FFffffff"/>
+        <color rgb="FFFFFFFF"/>
       </top>
       <bottom style="thin">
-        <color rgb="FFffff00"/>
+        <color rgb="FFFFFF00"/>
       </bottom>
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="16">
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="4" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="3" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="4" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="5" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="6" applyBorder="1" fontId="1" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="7" applyBorder="1" fontId="1" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="8" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="9" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="10" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
-  <cellStyles count="1">
-    <cellStyle xfId="0" builtinId="0" name="Normal"/>
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
-    <ext uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14ac:slicerStyles xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" defaultSlicerStyle="SlicerStyleLight1"/>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -530,10 +556,10 @@
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
-        <a:sysClr lastClr="000000" val="windowText"/>
+        <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr lastClr="FFFFFF" val="window"/>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="A7A7A7"/>
@@ -571,71 +597,71 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
-        <a:font typeface="맑은 고딕" script="Hang"/>
-        <a:font typeface="宋体" script="Hans"/>
-        <a:font typeface="新細明體" script="Hant"/>
-        <a:font typeface="Times New Roman" script="Arab"/>
-        <a:font typeface="Times New Roman" script="Hebr"/>
-        <a:font typeface="Tahoma" script="Thai"/>
-        <a:font typeface="Nyala" script="Ethi"/>
-        <a:font typeface="Vrinda" script="Beng"/>
-        <a:font typeface="Shruti" script="Gujr"/>
-        <a:font typeface="MoolBoran" script="Khmr"/>
-        <a:font typeface="Tunga" script="Knda"/>
-        <a:font typeface="Raavi" script="Guru"/>
-        <a:font typeface="Euphemia" script="Cans"/>
-        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
-        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
-        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
-        <a:font typeface="MV Boli" script="Thaa"/>
-        <a:font typeface="Mangal" script="Deva"/>
-        <a:font typeface="Gautami" script="Telu"/>
-        <a:font typeface="Latha" script="Taml"/>
-        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
-        <a:font typeface="Kalinga" script="Orya"/>
-        <a:font typeface="Kartika" script="Mlym"/>
-        <a:font typeface="DokChampa" script="Laoo"/>
-        <a:font typeface="Iskoola Pota" script="Sinh"/>
-        <a:font typeface="Mongolian Baiti" script="Mong"/>
-        <a:font typeface="Times New Roman" script="Viet"/>
-        <a:font typeface="Microsoft Uighur" script="Uigh"/>
-        <a:font typeface="Sylfaen" script="Geor"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
-        <a:font typeface="맑은 고딕" script="Hang"/>
-        <a:font typeface="宋体" script="Hans"/>
-        <a:font typeface="新細明體" script="Hant"/>
-        <a:font typeface="Arial" script="Arab"/>
-        <a:font typeface="Arial" script="Hebr"/>
-        <a:font typeface="Tahoma" script="Thai"/>
-        <a:font typeface="Nyala" script="Ethi"/>
-        <a:font typeface="Vrinda" script="Beng"/>
-        <a:font typeface="Shruti" script="Gujr"/>
-        <a:font typeface="DaunPenh" script="Khmr"/>
-        <a:font typeface="Tunga" script="Knda"/>
-        <a:font typeface="Raavi" script="Guru"/>
-        <a:font typeface="Euphemia" script="Cans"/>
-        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
-        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
-        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
-        <a:font typeface="MV Boli" script="Thaa"/>
-        <a:font typeface="Mangal" script="Deva"/>
-        <a:font typeface="Gautami" script="Telu"/>
-        <a:font typeface="Latha" script="Taml"/>
-        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
-        <a:font typeface="Kalinga" script="Orya"/>
-        <a:font typeface="Kartika" script="Mlym"/>
-        <a:font typeface="DokChampa" script="Laoo"/>
-        <a:font typeface="Iskoola Pota" script="Sinh"/>
-        <a:font typeface="Mongolian Baiti" script="Mong"/>
-        <a:font typeface="Arial" script="Viet"/>
-        <a:font typeface="Microsoft Uighur" script="Uigh"/>
-        <a:font typeface="Sylfaen" script="Geor"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -663,7 +689,7 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin scaled="1" ang="16200000"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
@@ -686,11 +712,11 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin scaled="1" ang="16200000"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="9525">
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr">
               <a:shade val="9500"/>
@@ -699,13 +725,13 @@
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="25400">
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="38100">
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -715,7 +741,7 @@
       <a:effectStyleLst>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="38000"/>
               </a:srgbClr>
@@ -724,7 +750,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -733,7 +759,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -741,10 +767,10 @@
           </a:effectLst>
           <a:scene3d>
             <a:camera prst="orthographicFront">
-              <a:rot rev="0" lon="0" lat="0"/>
+              <a:rot lat="0" lon="0" rev="0"/>
             </a:camera>
-            <a:lightRig dir="t" rig="threePt">
-              <a:rot rev="1200000" lon="0" lat="0"/>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
             </a:lightRig>
           </a:scene3d>
           <a:sp3d>
@@ -809,22 +835,22 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:F26"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:F27"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" style="15" width="25.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="15" width="32.57642857142857" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="15" width="16.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="15" width="15.719285714285713" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="15" width="12.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="15" width="19.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" width="25.7265625" style="12" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="32.54296875" style="12" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.7265625" style="12" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.7265625" style="12" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.54296875" style="12" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.7265625" style="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="19.5">
+    <row r="1" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -844,7 +870,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="19.5">
+    <row r="2" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>6</v>
       </c>
@@ -864,7 +890,7 @@
         <v>11</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="19.5">
+    <row r="3" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>12</v>
       </c>
@@ -884,7 +910,7 @@
         <v>11</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="19.5">
+    <row r="4" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>16</v>
       </c>
@@ -904,7 +930,7 @@
         <v>11</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="19.5">
+    <row r="5" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="5" t="s">
         <v>18</v>
       </c>
@@ -924,7 +950,7 @@
         <v>11</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="20.25">
+    <row r="6" spans="1:6" ht="20.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="6" t="s">
         <v>20</v>
       </c>
@@ -944,7 +970,7 @@
         <v>11</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="19.5">
+    <row r="7" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="9" t="s">
         <v>22</v>
       </c>
@@ -964,7 +990,7 @@
         <v>11</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="19.5">
+    <row r="8" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="6" t="s">
         <v>24</v>
       </c>
@@ -984,7 +1010,7 @@
         <v>11</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="19.5">
+    <row r="9" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="9" t="s">
         <v>26</v>
       </c>
@@ -1004,7 +1030,7 @@
         <v>11</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="19.5">
+    <row r="10" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="6" t="s">
         <v>28</v>
       </c>
@@ -1024,7 +1050,7 @@
         <v>11</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="20.25">
+    <row r="11" spans="1:6" ht="20.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="9" t="s">
         <v>30</v>
       </c>
@@ -1044,7 +1070,7 @@
         <v>11</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="17.25">
+    <row r="12" spans="1:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="12" t="s">
         <v>32</v>
       </c>
@@ -1064,7 +1090,7 @@
         <v>11</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="17.25">
+    <row r="13" spans="1:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="12" t="s">
         <v>34</v>
       </c>
@@ -1084,7 +1110,7 @@
         <v>11</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="17.25">
+    <row r="14" spans="1:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="12" t="s">
         <v>36</v>
       </c>
@@ -1104,7 +1130,7 @@
         <v>11</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="17.25">
+    <row r="15" spans="1:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="12" t="s">
         <v>38</v>
       </c>
@@ -1124,7 +1150,7 @@
         <v>11</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="17.25">
+    <row r="16" spans="1:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="12" t="s">
         <v>40</v>
       </c>
@@ -1144,7 +1170,7 @@
         <v>11</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="17.25">
+    <row r="17" spans="1:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="12" t="s">
         <v>42</v>
       </c>
@@ -1164,7 +1190,7 @@
         <v>11</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="17.25">
+    <row r="18" spans="1:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="12" t="s">
         <v>44</v>
       </c>
@@ -1184,7 +1210,7 @@
         <v>11</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="17.25">
+    <row r="19" spans="1:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="12" t="s">
         <v>46</v>
       </c>
@@ -1204,7 +1230,7 @@
         <v>11</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="17.25">
+    <row r="20" spans="1:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="12" t="s">
         <v>48</v>
       </c>
@@ -1224,7 +1250,7 @@
         <v>11</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="17.25">
+    <row r="21" spans="1:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="12" t="s">
         <v>50</v>
       </c>
@@ -1244,7 +1270,7 @@
         <v>11</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="17.25">
+    <row r="22" spans="1:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="12" t="s">
         <v>52</v>
       </c>
@@ -1264,7 +1290,7 @@
         <v>11</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="17.25">
+    <row r="23" spans="1:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="12" t="s">
         <v>54</v>
       </c>
@@ -1284,7 +1310,7 @@
         <v>11</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="17.25">
+    <row r="24" spans="1:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="12" t="s">
         <v>56</v>
       </c>
@@ -1304,7 +1330,7 @@
         <v>11</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="17.25">
+    <row r="25" spans="1:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="12" t="s">
         <v>58</v>
       </c>
@@ -1324,7 +1350,7 @@
         <v>11</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="18">
+    <row r="26" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" s="13" t="s">
         <v>60</v>
       </c>
@@ -1344,7 +1370,31 @@
         <v>11</v>
       </c>
     </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A27" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="B27" s="15" t="s">
+        <v>62</v>
+      </c>
+      <c r="C27" s="12" t="s">
+        <v>8</v>
+      </c>
+      <c r="D27" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="E27" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="F27" s="15" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B27" r:id="rId1" xr:uid="{5EDD04A9-91A1-4FF2-BABA-D3B3B7B99E8F}"/>
+    <hyperlink ref="F27" r:id="rId2" xr:uid="{E9DCBCF9-0E45-474B-A58B-A097033DE835}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
venue admin sorting + calendar loading fix
</commit_message>
<xml_diff>
--- a/user_info.xlsx
+++ b/user_info.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Aasthami\Documents\GitHub\VenueBookingSystem\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nehar\Web Dev\VenueBookingSystem\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E042163-7AA1-4444-A0D0-1CF373FCDAEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{396F2BE5-C981-42FD-9C9E-8B99617385FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="66">
   <si>
     <t>name</t>
   </si>
@@ -244,6 +244,15 @@
   </si>
   <si>
     <t>aastha.anuj.jajoo@gmail.com</t>
+  </si>
+  <si>
+    <t>Neha</t>
+  </si>
+  <si>
+    <t>neha.rathi2425@gmail.com</t>
+  </si>
+  <si>
+    <t>neharathi24180@gmail.com</t>
   </si>
 </sst>
 </file>
@@ -839,7 +848,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:F27"/>
+  <dimension ref="A1:F29"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="25.7265625" style="12" bestFit="1" customWidth="1"/>
@@ -1390,10 +1399,54 @@
         <v>11</v>
       </c>
     </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A28" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="B28" s="15" t="s">
+        <v>64</v>
+      </c>
+      <c r="C28" s="12" t="s">
+        <v>8</v>
+      </c>
+      <c r="D28" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="E28" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="F28" s="15" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A29" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="B29" s="15" t="s">
+        <v>65</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D29" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="E29" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="F29" s="15" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="B27" r:id="rId1" xr:uid="{5EDD04A9-91A1-4FF2-BABA-D3B3B7B99E8F}"/>
     <hyperlink ref="F27" r:id="rId2" xr:uid="{E9DCBCF9-0E45-474B-A58B-A097033DE835}"/>
+    <hyperlink ref="B28" r:id="rId3" xr:uid="{C38EF934-E449-4F4F-9815-0712C5B99636}"/>
+    <hyperlink ref="F28" r:id="rId4" xr:uid="{BE50F3E2-D7B6-44C1-A46D-70AD3265DCD6}"/>
+    <hyperlink ref="B29" r:id="rId5" xr:uid="{37956122-3151-4DB9-9600-01B1771FD8E5}"/>
+    <hyperlink ref="F29" r:id="rId6" xr:uid="{30966DC4-3476-46C6-B766-F649360C7350}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>